<commit_message>
Updated files for Testcases
</commit_message>
<xml_diff>
--- a/TestCase/Phone.xlsx
+++ b/TestCase/Phone.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\SDET_Wipro\TestCase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A054450-804C-4A65-A76C-CA7CD0BAC020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1616307A-EBD4-4713-9DAA-419065F31AFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4D67B6FC-63A5-4664-9C45-46C78102EF37}"/>
+    <workbookView xWindow="4005" yWindow="1290" windowWidth="15375" windowHeight="7875" xr2:uid="{4D67B6FC-63A5-4664-9C45-46C78102EF37}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="167">
   <si>
     <t>TC001</t>
   </si>
@@ -535,6 +535,12 @@
   </si>
   <si>
     <t>Phone should work smoothly without hanging</t>
+  </si>
+  <si>
+    <t>Torch</t>
+  </si>
+  <si>
+    <t>Baisc Function</t>
   </si>
 </sst>
 </file>
@@ -558,12 +564,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -593,7 +605,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -602,6 +614,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -918,7 +933,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C0A23B3-123D-46A5-A40A-79C5B10628A5}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -1426,28 +1441,28 @@
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+      <c r="A20" s="4">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="G20" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" s="4" t="s">
         <v>137</v>
       </c>
     </row>
@@ -1553,6 +1568,16 @@
       </c>
       <c r="H24" s="2" t="s">
         <v>164</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D27" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D28" s="1" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>